<commit_message>
Remove the 'Notes' sheet entirely from both templates
The real organization schema has no general-purpose free-text notes
field anywhere - the only 'notes' property in the whole schema is
edi.notes, specific to EDI transmission configuration, not a general
comment field. Every Notes-sheet row was always silently dropped
(never built into any output), so rather than keep collecting data
that goes nowhere, remove the sheet entirely from both blank templates,
both filled example workbooks, and both test fixtures.

Removed the now-pointless droppedNoteCount tracking from both
flatteners and both CLI scripts (the sheet no longer exists to read).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Organization_Template.xlsx
+++ b/Organization_Template.xlsx
@@ -15,8 +15,7 @@
     <sheet name="Contact people" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Interfaces" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Vendor info" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Notes" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Accounts" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Accounts" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -677,36 +676,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16.140625" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>NOTE</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Add URL notes/multi-category support and fix required-field highlighting
- Add a singular URL NOTE field (urls.notes) to both templates/example
  data, wired through both flatteners and RecordBuilder.
- Rename every CATEGORY column to CATEGORIES (it is a real array on
  every group that has it) and split category name lists on a
  dedicated ';' delimiter, independent of --list-delimiter.
- Audit required-field highlighting against the live FOLIO schemas:
  un-highlight Interfaces NAME (interface.json has no required fields
  at all) and Contact people EMAIL/PHONE (embedded groups are
  optional); highlight Interfaces USERNAME/PASSWORD as a required
  pair (interface_credential.json requires both together).
- Add the URLs sheet and ORG TYPE column that were missing from the
  blank Organization_Template.xlsx despite already existing in its
  example data and being documented in the README.
- Update tests and both READMEs accordingly.
</commit_message>
<xml_diff>
--- a/Organization_Template.xlsx
+++ b/Organization_Template.xlsx
@@ -12,10 +12,11 @@
     <sheet name="Addresses" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Phones" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Emails" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Contact people" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Interfaces" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Vendor info" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Accounts" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="URLs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Contact people" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Interfaces" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Vendor info" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Accounts" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -162,7 +163,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -220,6 +221,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -651,7 +656,7 @@
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>This applies on every sheet, not just Main Org record - e.g. PHONE on the Phones sheet, EMAIL on the Emails sheet, ACCOUNT NAME/ACCOUNT NUMBER/ACCOUNT STATUS on the Accounts sheet. One exception: an interface's USERNAME/PASSWORD (on the Interfaces sheet) aren't colored as mandatory since an interface doesn't need login credentials at all - but if you fill in either one, you must fill in both, or just that login-credentials record is skipped (the interface itself, and the rest of that organization, still build normally).</t>
+          <t>This applies on every sheet, not just Main Org record - e.g. PHONE on the Phones sheet, EMAIL on the Emails sheet, ACCOUNT NAME/ACCOUNT NUMBER/ACCOUNT STATUS on the Accounts sheet. A colored column can also be a 'required if you use this at all' pair rather than a plain single field: an interface's USERNAME/PASSWORD (on the Interfaces sheet) are both colored because if you fill in either one, you must fill in both, or just that login-credentials record is skipped (the interface itself, and the rest of that organization, still build normally). The Interfaces sheet's own NAME column, on the other hand, is intentionally NOT colored - the real FOLIO interface record has no required fields of its own, not even a name.</t>
         </is>
       </c>
     </row>
@@ -671,6 +676,96 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14.42578125" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>ORG CODE</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>PAYMENT METHOD</t>
+        </is>
+      </c>
+      <c r="C1" s="27" t="inlineStr">
+        <is>
+          <t>CURRENCIES</t>
+        </is>
+      </c>
+      <c r="D1" s="27" t="inlineStr">
+        <is>
+          <t>CLAIMING INTERVAL</t>
+        </is>
+      </c>
+      <c r="E1" s="27" t="inlineStr">
+        <is>
+          <t>DISCOUNT %</t>
+        </is>
+      </c>
+      <c r="F1" s="27" t="inlineStr">
+        <is>
+          <t>EXP ACTIVATION INTERVAL</t>
+        </is>
+      </c>
+      <c r="G1" s="27" t="inlineStr">
+        <is>
+          <t>EXP INVOICE INTERVAL</t>
+        </is>
+      </c>
+      <c r="H1" s="27" t="inlineStr">
+        <is>
+          <t>EXP RECEIPT INTERVAL</t>
+        </is>
+      </c>
+      <c r="I1" s="27" t="inlineStr">
+        <is>
+          <t>RENEWAL ACTIVATION INTERVAL</t>
+        </is>
+      </c>
+      <c r="J1" s="27" t="inlineStr">
+        <is>
+          <t>SUBSCRIPTION INTERVAL</t>
+        </is>
+      </c>
+      <c r="K1" s="27" t="inlineStr">
+        <is>
+          <t>EXPORT TO ACCOUNTING (Y/)</t>
+        </is>
+      </c>
+      <c r="L1" s="27" t="inlineStr">
+        <is>
+          <t>TAX ID</t>
+        </is>
+      </c>
+      <c r="M1" s="27" t="inlineStr">
+        <is>
+          <t>TAX %</t>
+        </is>
+      </c>
+      <c r="N1" s="27" t="inlineStr">
+        <is>
+          <t>LIABLE FOR VAT (Y/N)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -808,7 +903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S28"/>
+  <dimension ref="A1:T28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" style="8" min="1" max="1"/>
@@ -823,7 +918,8 @@
     <col width="17.5703125" customWidth="1" min="13" max="13"/>
     <col width="21.140625" customWidth="1" min="16" max="16"/>
     <col width="25" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -931,10 +1027,19 @@
       </c>
       <c r="R5" s="28" t="inlineStr">
         <is>
-          <t>URL CATEGORY</t>
-        </is>
-      </c>
-      <c r="S5" s="2" t="n"/>
+          <t>URL NOTE</t>
+        </is>
+      </c>
+      <c r="S5" s="28" t="inlineStr">
+        <is>
+          <t>URL CATEGORIES</t>
+        </is>
+      </c>
+      <c r="T5" s="28" t="inlineStr">
+        <is>
+          <t>ORG TYPE</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -1152,7 +1257,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>CATEGORY</t>
+          <t>CATEGORIES</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1298,7 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>CATEGORY</t>
+          <t>CATEGORIES</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1381,7 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>CATEGORY</t>
+          <t>CATEGORIES</t>
         </is>
       </c>
     </row>
@@ -1310,6 +1415,77 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18.140625" customWidth="1" min="1" max="1"/>
+    <col width="27.140625" customWidth="1" style="8" min="2" max="2"/>
+    <col width="27.140625" customWidth="1" min="3" max="3"/>
+    <col width="30" bestFit="1" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>ORG CODE</t>
+        </is>
+      </c>
+      <c r="B1" s="31" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>CATEGORIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>E.g., ebsco</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>customerservice@ebsco.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>E.g., ebsco</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>sales@ebsco.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1355,12 +1531,12 @@
           <t>NOTES</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="32" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">PHONE </t>
         </is>
@@ -1372,7 +1548,7 @@
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>CATEGORY</t>
+          <t>CATEGORIES</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1625,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1473,7 +1649,7 @@
           <t>ORG CODE</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="32" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
@@ -1493,12 +1669,12 @@
           <t>DELIVERY METHOD</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
         <is>
           <t>USERNAME</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="31" t="inlineStr">
         <is>
           <t>PASSWORD</t>
         </is>
@@ -1573,94 +1749,4 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14.42578125" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="45" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="27" t="inlineStr">
-        <is>
-          <t>PAYMENT METHOD</t>
-        </is>
-      </c>
-      <c r="C1" s="27" t="inlineStr">
-        <is>
-          <t>CURRENCIES</t>
-        </is>
-      </c>
-      <c r="D1" s="27" t="inlineStr">
-        <is>
-          <t>CLAIMING INTERVAL</t>
-        </is>
-      </c>
-      <c r="E1" s="27" t="inlineStr">
-        <is>
-          <t>DISCOUNT %</t>
-        </is>
-      </c>
-      <c r="F1" s="27" t="inlineStr">
-        <is>
-          <t>EXP ACTIVATION INTERVAL</t>
-        </is>
-      </c>
-      <c r="G1" s="27" t="inlineStr">
-        <is>
-          <t>EXP INVOICE INTERVAL</t>
-        </is>
-      </c>
-      <c r="H1" s="27" t="inlineStr">
-        <is>
-          <t>EXP RECEIPT INTERVAL</t>
-        </is>
-      </c>
-      <c r="I1" s="27" t="inlineStr">
-        <is>
-          <t>RENEWAL ACTIVATION INTERVAL</t>
-        </is>
-      </c>
-      <c r="J1" s="27" t="inlineStr">
-        <is>
-          <t>SUBSCRIPTION INTERVAL</t>
-        </is>
-      </c>
-      <c r="K1" s="27" t="inlineStr">
-        <is>
-          <t>EXPORT TO ACCOUNTING (Y/)</t>
-        </is>
-      </c>
-      <c r="L1" s="27" t="inlineStr">
-        <is>
-          <t>TAX ID</t>
-        </is>
-      </c>
-      <c r="M1" s="27" t="inlineStr">
-        <is>
-          <t>TAX %</t>
-        </is>
-      </c>
-      <c r="N1" s="27" t="inlineStr">
-        <is>
-          <t>LIABLE FOR VAT (Y/N)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>